<commit_message>
Switch investor emails to the short version (about 120 words)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2WBTUaYVg19XogRfpJJ3d
</commit_message>
<xml_diff>
--- a/collateral/SimReal-海外VC名单.xlsx
+++ b/collateral/SimReal-海外VC名单.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Your State of AI Report tracks the shift to RL post-training, and Air Street backs AI-first companies from seed; SimReal builds the RL environments and verifiers that shift runs on, starting with finance.</t>
+          <t>Your State of AI Report tracks the shift to RL post-training, and Air Street backs AI-first companies from seed; we're building for that shift, starting with finance.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -639,19 +639,16 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
           <t>Hi Nathan,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
-Your State of AI Report tracks the shift to RL post-training, and Air Street backs AI-first companies from seed; SimReal builds the RL environments and verifiers that shift runs on, starting with finance.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
+Your State of AI Report tracks the shift to RL post-training, and Air Street backs AI-first companies from seed; we're building for that shift, starting with finance.
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -740,19 +737,16 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
           <t>Hi Sarah,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 Conviction led Trajectory's seed for continual learning in May; we build the finance environments where that kind of learning gets scored against real outcomes.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -841,19 +835,16 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
           <t>Hi Vijay,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 Mayfield backed Bespoke Labs on the view that agents depend on data, environments and evaluation; we build all three for finance, from trading to month-end close.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -942,19 +933,16 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
           <t>Hi Kanyi,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 Kindred led Scorecard's seed to test AI agents across thousands of simulated scenarios; we build the environments and verifiers that train those agents, starting with finance.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1043,19 +1031,16 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
           <t>Hi Lu,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 You led AgileRL's seed calling reinforcement learning the gold standard of AI training; we build the finance environments and verifiers that make RL work outside the lab.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1144,19 +1129,16 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
           <t>Hi Andy,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 Laude described backing Arena as turning research-driven evaluation into AI infrastructure; we're doing that for finance, where models are scored by real market outcomes.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1245,19 +1227,16 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
           <t>Hi Vivek,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 You co-led Gray Swan's Series A after hearing a chorus of praise from frontier labs; we sell those same labs RL environments and verifiers, starting with finance.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1346,19 +1325,16 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
           <t>Hi Deedy,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 Your July map counted 50+ companies selling data and RL environments to labs, with most revenue in four players; we're a finance-specialist entrant with quant founders and our own experts.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1447,19 +1423,16 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
           <t>Hi Jeremy,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 The House Fund backed Veris AI's seed for simulated environments that train enterprise agents; we build those environments for finance.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1548,19 +1521,16 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
           <t>Hi Chris,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 Your RL environments piece argued verification, not model capability, is what makes automation durable; verifiers are the core of what we build for finance.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1649,19 +1619,16 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
           <t>Hi Hadley,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 Eniac joined Origin Lab's seed to turn game worlds into AI training data; we turn financial markets into RL environments for the same labs.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1750,19 +1717,16 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
           <t>Hi Grace,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 Lux backed Applied Compute twice as enterprises start training their own models; we supply the RL environments and expert data those runs need, starting with finance and accounting.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1851,19 +1815,16 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
           <t>Hi Jared,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 TRV has been hosting AI x Wall Street and AI-agent events for the trading world; we're ex-quants building RL environments that train agents on real market data.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -1952,19 +1913,16 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
           <t>Hi Yuri,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 You led Arga's seed and argued that repeatable sandboxes matter even more for agents; we've built that for finance, where outcomes settle in real markets.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal
@@ -2049,19 +2007,16 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>SimReal: RL environments where AI learns from real outcomes (seed)</t>
+          <t>SimReal: RL environments for finance, built by ex-Jane Street and Citadel quants (seed)</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
           <t>Hi HRT Ventures team,
-I'm [Your name], co-founder of SimReal (simreal.co). We build the environments where AI does real work, is scored by real outcomes, and trains on those outcomes.
+I'm [Your name], co-founder of SimReal (simreal.co). We build RL environments and verifiers where models do real work and are scored on real outcomes.
 HRT Ventures joined Vals AI's Series A in August; we build trading RL environments, and our founders come from the same quant world.
-- Team: four quants from Cambridge, LSE and Duke, with backgrounds at Jane Street, Citadel, D. E. Shaw, Millennium and Optiver. All four turned down return offers.
-- Proof: our trading environment, Xitadel, improved Qwen3.8-27B's trading performance by 12% on unseen market data, reproduced across independent runs. On its public preview the best frontier model scores 77.3 against a human reference of 80.
-- Speed: seven products in our first 14 days with no outside capital; 500+ GitHub stars in week one.
-- Commercial: in talks with two frontier labs; already working with Surge AI and AfterQuery; 7,000+ experts signed up and 200,000+ professionals reachable through 21 partner universities.
-We're raising a $20M seed and are in conversations with tier-1 funds. Can I send you the deck, or find 30 minutes next week?
+Our trading environment, Xitadel, lifted Qwen3.8-27B's trading performance 12% on unseen market data, reproduced across independent runs. We already supply Surge AI and AfterQuery, and 7,000+ domain experts have signed up. We're four quants from Jane Street, Citadel, Millennium and Optiver (Cambridge, LSE, Duke), raising a $20M seed and in conversations with tier-1 funds.
+Worth 20 minutes? Happy to send the deck.
 Best,
 [Your name]
 Co-founder, SimReal

</xml_diff>